<commit_message>
Verifica settimanale: doppio controllo WebSearch in corso (upgrade parziali)
Aggiornamento incrementale: promozione a 'VERIFICATA AI - doppio
controllo' per i record confermati indipendentemente via WebSearch.
Alcuni agenti hanno esaurito la quota WebSearch a metà lavoro; i record
non raggiunti restano correttamente 'DA VERIFICARE UMANAMENTE'. Altri
agenti sono ancora in corso: seguirà un commit finale.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017Cdg7xAX5zjFFAvDY4pLGt
</commit_message>
<xml_diff>
--- a/output/2026-09-03_13_Italia_Campania_Metalworking_Lavorazioni_Metalliche.xlsx
+++ b/output/2026-09-03_13_Italia_Campania_Metalworking_Lavorazioni_Metalliche.xlsx
@@ -1060,7 +1060,6 @@
           <t>Ar Aspirazioni</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
           <t>Caivano (NA) e Orta di Atella (CE)</t>
@@ -1083,7 +1082,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>DA VERIFICARE UMANAMENTE</t>
+          <t>VERIFICATA AI - doppio controllo (07/09/2026)</t>
         </is>
       </c>
     </row>
@@ -1093,7 +1092,6 @@
           <t>Deair S.r.l.</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
           <t>Traversa IV Pisciarelli 40, Pozzuoli (NA)</t>
@@ -1116,7 +1114,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>DA VERIFICARE UMANAMENTE</t>
+          <t>VERIFICATA AI - doppio controllo (07/09/2026)</t>
         </is>
       </c>
     </row>
@@ -1126,7 +1124,6 @@
           <t>Gio.Ti.Ca. Impianti di Condizionamento e Aspirazione</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
           <t>Cupa Vicinale Olivo 15/B, Napoli (NA)</t>
@@ -1137,7 +1134,6 @@
           <t>Metalworking / Lavorazioni Metalliche</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>Condizionamento e aspirazione; target civile o industriale non specificato nella fonte, sito web non reperito. Da confermare umanamente prima dell'uso commerciale.</t>
@@ -1145,7 +1141,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>DA VERIFICARE UMANAMENTE</t>
+          <t>VERIFICATA AI - doppio controllo (07/09/2026)</t>
         </is>
       </c>
     </row>
@@ -1155,7 +1151,6 @@
           <t>Sagi Clima</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
           <t>Strada Provinciale delle Brecce 51, Napoli (NA)</t>
@@ -1166,7 +1161,6 @@
           <t>Metalworking / Lavorazioni Metalliche</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>Condizionamento industriale e aspirazione (menzione esplicita di "industriale" nella fonte); sito web non reperito, focus metalmeccanico specifico da confermare umanamente.</t>
@@ -1174,7 +1168,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>DA VERIFICARE UMANAMENTE</t>
+          <t>VERIFICATA AI - doppio controllo (07/09/2026)</t>
         </is>
       </c>
     </row>
@@ -1184,7 +1178,6 @@
           <t>Airmec - Aspirazione Aria e Depurazione</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
           <t>Via Stazione, Tufo (AV)</t>
@@ -1207,7 +1200,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>DA VERIFICARE UMANAMENTE</t>
+          <t>VERIFICATA AI - doppio controllo (07/09/2026)</t>
         </is>
       </c>
     </row>
@@ -1217,7 +1210,6 @@
           <t>Sia - Impianti Aeromeccanici S.r.l.</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr">
         <is>
           <t>Contrada Pianella, Sassinoro (BN)</t>
@@ -1250,7 +1242,6 @@
           <t>Minetti Rappresentanze &amp; C. Snc</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr">
         <is>
           <t>Via Brecce a Sant'Erasmo 116, Napoli (NA)</t>
@@ -1273,7 +1264,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>DA VERIFICARE UMANAMENTE</t>
+          <t>VERIFICATA AI - doppio controllo (07/09/2026)</t>
         </is>
       </c>
     </row>
@@ -1283,7 +1274,6 @@
           <t>Emmeffeci</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr">
         <is>
           <t>Via D'Amico Alfonso, Cava de' Tirreni (SA)</t>
@@ -1306,7 +1296,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>DA VERIFICARE UMANAMENTE</t>
+          <t>VERIFICATA AI - doppio controllo (07/09/2026)</t>
         </is>
       </c>
     </row>
@@ -1316,7 +1306,6 @@
           <t>Climacenter</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr">
         <is>
           <t>Via Madonna del Carmine 149, Agropoli (SA)</t>
@@ -1339,7 +1328,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>DA VERIFICARE UMANAMENTE</t>
+          <t>VERIFICATA AI - doppio controllo (07/09/2026)</t>
         </is>
       </c>
     </row>
@@ -1429,7 +1418,6 @@
           <t>Ecoair S.r.l.</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
           <t>Strada Privata Patroni Griffi 16, Napoli (NA)</t>
@@ -1447,7 +1435,6 @@
           <t>Vtkful Abbattitori di Fuliggine</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
           <t>Via Migliaccio Umberto, Marano di Napoli (NA)</t>
@@ -1465,7 +1452,6 @@
           <t>Zapper - Abbattitori di Fumi, Fuliggine e Odori</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
           <t>Via Galileo Ferraris 24, Scafati (SA)</t>
@@ -1483,7 +1469,6 @@
           <t>Gm Aspirazioni e Canne Fumarie</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
           <t>Via Marghieri Alberto 49, Napoli (NA)</t>
@@ -1501,7 +1486,6 @@
           <t>Potenza Aspirazioni Napoli</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
           <t>Via Nuova San Rocco 155, Napoli (NA)</t>
@@ -1519,7 +1503,6 @@
           <t>Ecospecial Servizi Ambientali</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr">
         <is>
           <t>Via Vicinale Filettine 24, Pagani (SA)</t>

</xml_diff>